<commit_message>
Update Paneer Combo price to 349 and regenerate all HTML, Excel, and PDF menus
</commit_message>
<xml_diff>
--- a/Hotel_Sky5_Market_Pricing_Audit.xlsx
+++ b/Hotel_Sky5_Market_Pricing_Audit.xlsx
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1781,14 +1781,14 @@
       </c>
       <c r="B39" s="20" t="inlineStr">
         <is>
-          <t>Non-Veg Deluxe Thali</t>
+          <t>Paneer Combo</t>
         </is>
       </c>
       <c r="C39" s="21" t="n">
-        <v>499</v>
+        <v>349</v>
       </c>
       <c r="D39" s="21" t="n">
-        <v>504</v>
+        <v>354</v>
       </c>
       <c r="E39" s="21">
         <f>D39-C39</f>
@@ -1807,19 +1807,19 @@
     <row r="40" ht="20.1" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
         <is>
-          <t>Desserts</t>
+          <t>Combos &amp; Thalis</t>
         </is>
       </c>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>Gulab Jamun (2 pcs)</t>
+          <t>Butter Chicken Combo</t>
         </is>
       </c>
       <c r="C40" s="21" t="n">
-        <v>109</v>
+        <v>449</v>
       </c>
       <c r="D40" s="21" t="n">
-        <v>114</v>
+        <v>454</v>
       </c>
       <c r="E40" s="21">
         <f>D40-C40</f>
@@ -1831,26 +1831,26 @@
       </c>
       <c r="G40" s="23" t="inlineStr">
         <is>
-          <t>Sweet Upsell</t>
+          <t>High Value Combo</t>
         </is>
       </c>
     </row>
     <row r="41" ht="20.1" customHeight="1">
       <c r="A41" s="19" t="inlineStr">
         <is>
-          <t>Desserts</t>
+          <t>Combos &amp; Thalis</t>
         </is>
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
-          <t>Kulfi</t>
+          <t>Non-Veg Deluxe Thali</t>
         </is>
       </c>
       <c r="C41" s="21" t="n">
-        <v>99</v>
+        <v>499</v>
       </c>
       <c r="D41" s="21" t="n">
-        <v>104</v>
+        <v>504</v>
       </c>
       <c r="E41" s="21">
         <f>D41-C41</f>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="G41" s="23" t="inlineStr">
         <is>
-          <t>Sweet Upsell</t>
+          <t>High Value Combo</t>
         </is>
       </c>
     </row>
@@ -1874,14 +1874,14 @@
       </c>
       <c r="B42" s="20" t="inlineStr">
         <is>
-          <t>Ice Cream (Single Scoop)</t>
+          <t>Gulab Jamun (2 pcs)</t>
         </is>
       </c>
       <c r="C42" s="21" t="n">
-        <v>99</v>
+        <v>109</v>
       </c>
       <c r="D42" s="21" t="n">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="E42" s="21">
         <f>D42-C42</f>
@@ -1905,14 +1905,14 @@
       </c>
       <c r="B43" s="20" t="inlineStr">
         <is>
-          <t>Ice Cream (Double Scoop)</t>
+          <t>Kulfi</t>
         </is>
       </c>
       <c r="C43" s="21" t="n">
-        <v>169</v>
+        <v>99</v>
       </c>
       <c r="D43" s="21" t="n">
-        <v>174</v>
+        <v>104</v>
       </c>
       <c r="E43" s="21">
         <f>D43-C43</f>
@@ -1931,19 +1931,19 @@
     <row r="44" ht="20.1" customHeight="1">
       <c r="A44" s="19" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Desserts</t>
         </is>
       </c>
       <c r="B44" s="20" t="inlineStr">
         <is>
-          <t>Tea</t>
+          <t>Ice Cream (Single Scoop)</t>
         </is>
       </c>
       <c r="C44" s="21" t="n">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="D44" s="21" t="n">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="E44" s="21">
         <f>D44-C44</f>
@@ -1955,26 +1955,26 @@
       </c>
       <c r="G44" s="23" t="inlineStr">
         <is>
-          <t>High Frequency Item</t>
+          <t>Sweet Upsell</t>
         </is>
       </c>
     </row>
     <row r="45" ht="20.1" customHeight="1">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>Beverages</t>
+          <t>Desserts</t>
         </is>
       </c>
       <c r="B45" s="20" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Ice Cream (Double Scoop)</t>
         </is>
       </c>
       <c r="C45" s="21" t="n">
-        <v>70</v>
+        <v>169</v>
       </c>
       <c r="D45" s="21" t="n">
-        <v>75</v>
+        <v>174</v>
       </c>
       <c r="E45" s="21">
         <f>D45-C45</f>
@@ -1986,7 +1986,7 @@
       </c>
       <c r="G45" s="23" t="inlineStr">
         <is>
-          <t>High Frequency Item</t>
+          <t>Sweet Upsell</t>
         </is>
       </c>
     </row>
@@ -1998,14 +1998,14 @@
       </c>
       <c r="B46" s="20" t="inlineStr">
         <is>
-          <t>Glass of Milk</t>
+          <t>Tea</t>
         </is>
       </c>
       <c r="C46" s="21" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D46" s="21" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E46" s="21">
         <f>D46-C46</f>
@@ -2029,14 +2029,14 @@
       </c>
       <c r="B47" s="20" t="inlineStr">
         <is>
-          <t>Lemon Water</t>
+          <t>Coffee</t>
         </is>
       </c>
       <c r="C47" s="21" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D47" s="21" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="E47" s="21">
         <f>D47-C47</f>
@@ -2060,14 +2060,14 @@
       </c>
       <c r="B48" s="20" t="inlineStr">
         <is>
-          <t>Fresh Lemonade</t>
+          <t>Glass of Milk</t>
         </is>
       </c>
       <c r="C48" s="21" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="D48" s="21" t="n">
-        <v>104</v>
+        <v>75</v>
       </c>
       <c r="E48" s="21">
         <f>D48-C48</f>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="B49" s="20" t="inlineStr">
         <is>
-          <t>Plain Soda</t>
+          <t>Lemon Water</t>
         </is>
       </c>
       <c r="C49" s="21" t="n">
@@ -2122,14 +2122,14 @@
       </c>
       <c r="B50" s="20" t="inlineStr">
         <is>
-          <t>Sweet Lassi</t>
+          <t>Fresh Lemonade</t>
         </is>
       </c>
       <c r="C50" s="21" t="n">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="D50" s="21" t="n">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="E50" s="21">
         <f>D50-C50</f>
@@ -2153,14 +2153,14 @@
       </c>
       <c r="B51" s="20" t="inlineStr">
         <is>
-          <t>Salted Lassi</t>
+          <t>Plain Soda</t>
         </is>
       </c>
       <c r="C51" s="21" t="n">
-        <v>109</v>
+        <v>50</v>
       </c>
       <c r="D51" s="21" t="n">
-        <v>114</v>
+        <v>55</v>
       </c>
       <c r="E51" s="21">
         <f>D51-C51</f>
@@ -2184,14 +2184,14 @@
       </c>
       <c r="B52" s="20" t="inlineStr">
         <is>
-          <t>Coke</t>
+          <t>Sweet Lassi</t>
         </is>
       </c>
       <c r="C52" s="21" t="n">
-        <v>50</v>
+        <v>109</v>
       </c>
       <c r="D52" s="21" t="n">
-        <v>55</v>
+        <v>114</v>
       </c>
       <c r="E52" s="21">
         <f>D52-C52</f>
@@ -2215,14 +2215,14 @@
       </c>
       <c r="B53" s="20" t="inlineStr">
         <is>
-          <t>Limca</t>
+          <t>Salted Lassi</t>
         </is>
       </c>
       <c r="C53" s="21" t="n">
-        <v>50</v>
+        <v>109</v>
       </c>
       <c r="D53" s="21" t="n">
-        <v>55</v>
+        <v>114</v>
       </c>
       <c r="E53" s="21">
         <f>D53-C53</f>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B54" s="20" t="inlineStr">
         <is>
-          <t>Mineral Water (1 Ltr)</t>
+          <t>Coke</t>
         </is>
       </c>
       <c r="C54" s="21" t="n">
@@ -2270,29 +2270,91 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="15" t="inlineStr">
+      <c r="A55" s="19" t="inlineStr">
+        <is>
+          <t>Beverages</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="inlineStr">
+        <is>
+          <t>Limca</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="D55" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="E55" s="21">
+        <f>D55-C55</f>
+        <v/>
+      </c>
+      <c r="F55" s="22">
+        <f>E55/D55</f>
+        <v/>
+      </c>
+      <c r="G55" s="23" t="inlineStr">
+        <is>
+          <t>High Frequency Item</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="19" t="inlineStr">
+        <is>
+          <t>Beverages</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="inlineStr">
+        <is>
+          <t>Mineral Water (1 Ltr)</t>
+        </is>
+      </c>
+      <c r="C56" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="D56" s="21" t="n">
+        <v>55</v>
+      </c>
+      <c r="E56" s="21">
+        <f>D56-C56</f>
+        <v/>
+      </c>
+      <c r="F56" s="22">
+        <f>E56/D56</f>
+        <v/>
+      </c>
+      <c r="G56" s="23" t="inlineStr">
+        <is>
+          <t>High Frequency Item</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="B55" s="16" t="n"/>
-      <c r="C55" s="17">
-        <f>AVERAGE(C2:C54)</f>
-        <v/>
-      </c>
-      <c r="D55" s="17">
-        <f>AVERAGE(D2:D54)</f>
-        <v/>
-      </c>
-      <c r="E55" s="17">
-        <f>AVERAGE(E2:E54)</f>
-        <v/>
-      </c>
-      <c r="F55" s="24">
-        <f>AVERAGE(F2:F54)</f>
-        <v/>
-      </c>
-      <c r="G55" s="16" t="n"/>
+      <c r="B57" s="16" t="n"/>
+      <c r="C57" s="17">
+        <f>AVERAGE(C2:C56)</f>
+        <v/>
+      </c>
+      <c r="D57" s="17">
+        <f>AVERAGE(D2:D56)</f>
+        <v/>
+      </c>
+      <c r="E57" s="17">
+        <f>AVERAGE(E2:E56)</f>
+        <v/>
+      </c>
+      <c r="F57" s="24">
+        <f>AVERAGE(F2:F56)</f>
+        <v/>
+      </c>
+      <c r="G57" s="16" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Restore Paneer Combo and Butter Chicken Combo, update descriptions of Veg/Paneer/Chicken combos with pickles and rice/roti adjustments as per notes
</commit_message>
<xml_diff>
--- a/Hotel_Sky5_Market_Pricing_Audit.xlsx
+++ b/Hotel_Sky5_Market_Pricing_Audit.xlsx
@@ -1785,10 +1785,10 @@
         </is>
       </c>
       <c r="C39" s="21" t="n">
-        <v>349</v>
+        <v>249</v>
       </c>
       <c r="D39" s="21" t="n">
-        <v>354</v>
+        <v>254</v>
       </c>
       <c r="E39" s="21">
         <f>D39-C39</f>

</xml_diff>